<commit_message>
feat(battle): add participant prefab configuration
</commit_message>
<xml_diff>
--- a/DataTables/Datas/battle.enemy.xlsx
+++ b/DataTables/Datas/battle.enemy.xlsx
@@ -433,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4CF470-E9E0-44FF-BA6C-71B5C42FB7B2}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.75" bestFit="1" customWidth="1"/>
@@ -450,14 +450,21 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name_i18n_key</t>
+        </is>
       </c>
       <c r="D1" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>view_prefab_address</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -476,6 +483,11 @@
       <c r="E2" t="s">
         <v>6</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -489,28 +501,42 @@
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
-        <v>11</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Name i18n key</t>
+        </is>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>View Prefab Address</t>
+        </is>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B5">
         <v>2001</v>
       </c>
-      <c r="C5" t="s">
-        <v>14</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>battle.enemy.test_slime.name</t>
+        </is>
       </c>
       <c r="D5">
         <v>20</v>
       </c>
       <c r="E5">
         <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Assets/Arts/Runtime/Character/Prefabs/pfb_char_enemy.prefab</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(config): use logical keys for character assets
</commit_message>
<xml_diff>
--- a/DataTables/Datas/battle.enemy.xlsx
+++ b/DataTables/Datas/battle.enemy.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6cb684c1938241eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R94eecbcb7cf84f56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -479,10 +479,8 @@
       <x:c r="E1" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">view_prefab_address</x:t>
-        </x:is>
+      <x:c r="F1" s="1" t="str">
+        <x:v>view_prefab_key</x:v>
       </x:c>
       <x:c r="G1" s="12" t="str">
         <x:v>behavior_group_id</x:v>
@@ -537,10 +535,8 @@
       <x:c r="E4" s="4" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F4" s="4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">View Prefab Address</x:t>
-        </x:is>
+      <x:c r="F4" s="4" t="str">
+        <x:v>View Prefab Key</x:v>
       </x:c>
       <x:c r="G4" s="14" t="str">
         <x:v>Behavior group ID</x:v>
@@ -561,10 +557,8 @@
       <x:c r="E5" s="9">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F5" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Assets/Arts/Runtime/Character/Prefabs/pfb_char_enemy.prefab</x:t>
-        </x:is>
+      <x:c r="F5" s="10" t="str">
+        <x:v>pfb_char_enemy</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
         <x:v>6001</x:v>
@@ -585,7 +579,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Assets/Arts/Runtime/Character/Prefabs/pfb_char_enemy.prefab</x:v>
+        <x:v>pfb_char_enemy</x:v>
       </x:c>
       <x:c r="G6" s="16" t="n">
         <x:v>6002</x:v>

</xml_diff>